<commit_message>
Modified with XLOOKUP queries
</commit_message>
<xml_diff>
--- a/XLOOKUP VS VLOOKUP.xlsx
+++ b/XLOOKUP VS VLOOKUP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24701"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/579481080490e445/Documents/Excel Series Excels/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Previous\programming\DA\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{625F3FEF-17C5-43E2-BFC2-A4868BFCBA3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2710DD79-32A6-47C9-902A-0857C1FEBFB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5EA44D8F-79D3-45F5-A0F6-C7F47358B7ED}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5EA44D8F-79D3-45F5-A0F6-C7F47358B7ED}"/>
   </bookViews>
   <sheets>
     <sheet name="XLookUp" sheetId="1" r:id="rId1"/>
@@ -39,8 +39,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="97">
   <si>
     <t>EmployeeID</t>
   </si>
@@ -316,6 +338,21 @@
   </si>
   <si>
     <t>Address</t>
+  </si>
+  <si>
+    <t xml:space="preserve">using last name </t>
+  </si>
+  <si>
+    <t>using first name</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> last to first </t>
+  </si>
+  <si>
+    <t>first to last</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exact or next larger </t>
   </si>
 </sst>
 </file>
@@ -373,9 +410,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -413,7 +450,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -519,7 +556,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -661,7 +698,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -670,15 +707,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1027015F-D30F-450C-928C-DE78480974B7}">
   <dimension ref="A1:P23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="24.5546875" customWidth="1"/>
-    <col min="8" max="8" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="40.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.26953125" customWidth="1"/>
+    <col min="2" max="2" width="24.54296875" customWidth="1"/>
+    <col min="8" max="8" width="14.6328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="40.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
       <c r="E1" t="s">
         <v>0</v>
       </c>
@@ -716,7 +754,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>60</v>
       </c>
@@ -757,10 +795,14 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>65</v>
       </c>
+      <c r="B3" t="str">
+        <f>_xlfn.XLOOKUP(A3,H2:H10,P2:P10)</f>
+        <v>Toby.Flenderson@DunderMifflinCorporate.com</v>
+      </c>
       <c r="E3">
         <v>1002</v>
       </c>
@@ -795,10 +837,14 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>62</v>
       </c>
+      <c r="B4" t="str">
+        <f>_xlfn.XLOOKUP(A4,H3:H11,P3:P11)</f>
+        <v>Pam.Beasley@DunderMifflin.com</v>
+      </c>
       <c r="E4">
         <v>1003</v>
       </c>
@@ -833,10 +879,14 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>67</v>
       </c>
+      <c r="B5" t="str">
+        <f>_xlfn.XLOOKUP(A5,H4:H12,P4:P12)</f>
+        <v>Meredith.Palmer@Yahoo.com</v>
+      </c>
       <c r="E5">
         <v>1004</v>
       </c>
@@ -871,10 +921,14 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>69</v>
       </c>
+      <c r="B6" t="str">
+        <f>_xlfn.XLOOKUP(A6,H5:H13,P5:P13)</f>
+        <v>Kevin.Malone@DunderMifflin.com</v>
+      </c>
       <c r="E6">
         <v>1005</v>
       </c>
@@ -909,7 +963,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="E7">
         <v>1006</v>
       </c>
@@ -944,7 +998,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="E8">
         <v>1007</v>
       </c>
@@ -979,7 +1033,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="E9">
         <v>1008</v>
       </c>
@@ -1014,7 +1068,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="E10">
         <v>1009</v>
       </c>
@@ -1049,15 +1103,15 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="8:8" x14ac:dyDescent="0.35">
       <c r="H22" t="str">
-        <f t="shared" ref="H22:H23" si="0">CONCATENATE(F12," ",G12)</f>
+        <f>CONCATENATE(F12," ",G12)</f>
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="23" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="8:8" x14ac:dyDescent="0.35">
       <c r="H23" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(F13," ",G13)</f>
         <v xml:space="preserve"> </v>
       </c>
     </row>
@@ -1069,16 +1123,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEFF05A7-3704-402E-8684-C856D6F82881}">
   <dimension ref="A1:P23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5546875" customWidth="1"/>
-    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="40.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="33.7265625" customWidth="1"/>
+    <col min="9" max="9" width="14.6328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="40.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
       <c r="F1" t="s">
         <v>0</v>
       </c>
@@ -1113,7 +1168,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>60</v>
       </c>
@@ -1157,10 +1212,17 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>65</v>
       </c>
+      <c r="B3" t="str" cm="1">
+        <f t="array" ref="B3:C3">_xlfn.XLOOKUP(A3,I2:I10,O2:P10)</f>
+        <v>8/30/2017</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Toby.Flenderson@DunderMifflinCorporate.com</v>
+      </c>
       <c r="F3">
         <v>1002</v>
       </c>
@@ -1195,10 +1257,17 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>62</v>
       </c>
+      <c r="B4" t="str" cm="1">
+        <f t="array" ref="B4:C4">_xlfn.XLOOKUP(A4,I3:I11,O3:P11)</f>
+        <v>10/10/2015</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Pam.Beasley@DunderMifflin.com</v>
+      </c>
       <c r="F4">
         <v>1003</v>
       </c>
@@ -1233,10 +1302,17 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>67</v>
       </c>
+      <c r="B5" t="str" cm="1">
+        <f t="array" ref="B5:C5">_xlfn.XLOOKUP(A5,I4:I12,O4:P12)</f>
+        <v>9/11/2013</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Meredith.Palmer@Yahoo.com</v>
+      </c>
       <c r="F5">
         <v>1004</v>
       </c>
@@ -1271,10 +1347,17 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>69</v>
       </c>
+      <c r="B6" t="str" cm="1">
+        <f t="array" ref="B6:C6">_xlfn.XLOOKUP(A6,I5:I13,O5:P13)</f>
+        <v>4/22/2015</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Kevin.Malone@DunderMifflin.com</v>
+      </c>
       <c r="F6">
         <v>1005</v>
       </c>
@@ -1309,7 +1392,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="F7">
         <v>1006</v>
       </c>
@@ -1344,7 +1427,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="F8">
         <v>1007</v>
       </c>
@@ -1379,7 +1462,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="F9">
         <v>1008</v>
       </c>
@@ -1414,7 +1497,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="F10">
         <v>1009</v>
       </c>
@@ -1449,15 +1532,15 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="9:9" x14ac:dyDescent="0.35">
       <c r="I22" t="str">
-        <f t="shared" ref="I22:I23" si="0">CONCATENATE(G12," ",H12)</f>
+        <f>CONCATENATE(G12," ",H12)</f>
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="23" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="9:9" x14ac:dyDescent="0.35">
       <c r="I23" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(G13," ",H13)</f>
         <v xml:space="preserve"> </v>
       </c>
     </row>
@@ -1469,16 +1552,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32A7D64C-38C9-4586-AD37-471BFBE38708}">
   <dimension ref="A1:O23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.5546875" customWidth="1"/>
-    <col min="8" max="8" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="40.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.81640625" customWidth="1"/>
+    <col min="3" max="3" width="15.7265625" customWidth="1"/>
+    <col min="8" max="8" width="14.6328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="40.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="E1" t="s">
         <v>0</v>
       </c>
@@ -1513,7 +1597,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>60</v>
       </c>
@@ -1554,10 +1638,14 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>86</v>
       </c>
+      <c r="B3" t="str">
+        <f>_xlfn.XLOOKUP(A3,H2:H10,O2:O10,"Not Found")</f>
+        <v>Not Found</v>
+      </c>
       <c r="E3">
         <v>1002</v>
       </c>
@@ -1592,10 +1680,17 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>18</v>
       </c>
+      <c r="B4" t="str">
+        <f>_xlfn.XLOOKUP("*"&amp;A4,H2:H10,O2:O10,"Not Found",2)</f>
+        <v>Pam.Beasley@DunderMifflin.com</v>
+      </c>
+      <c r="C4" t="s">
+        <v>92</v>
+      </c>
       <c r="E4">
         <v>1003</v>
       </c>
@@ -1630,10 +1725,17 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>46</v>
       </c>
+      <c r="B5" t="str">
+        <f>_xlfn.XLOOKUP(A5&amp;"*",H2:H10,O2:O10,"Not Found",2)</f>
+        <v>Meredith.Palmer@Yahoo.com</v>
+      </c>
+      <c r="C5" t="s">
+        <v>93</v>
+      </c>
       <c r="E5">
         <v>1004</v>
       </c>
@@ -1668,10 +1770,17 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>87</v>
       </c>
+      <c r="B6" t="str">
+        <f>_xlfn.XLOOKUP(A6&amp;"*",H3:H11,O3:O11,"Not Found",2)</f>
+        <v>Kevin.Malone@DunderMifflin.com</v>
+      </c>
+      <c r="C6" t="s">
+        <v>93</v>
+      </c>
       <c r="E6">
         <v>1005</v>
       </c>
@@ -1706,7 +1815,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="E7">
         <v>1006</v>
       </c>
@@ -1741,7 +1850,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="E8">
         <v>1007</v>
       </c>
@@ -1776,7 +1885,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="E9">
         <v>1008</v>
       </c>
@@ -1811,7 +1920,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="E10">
         <v>1009</v>
       </c>
@@ -1846,15 +1955,15 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="8:8" x14ac:dyDescent="0.35">
       <c r="H22" t="str">
-        <f t="shared" ref="H22:H23" si="0">CONCATENATE(F12," ",G12)</f>
+        <f>CONCATENATE(F12," ",G12)</f>
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="23" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="8:8" x14ac:dyDescent="0.35">
       <c r="H23" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(F13," ",G13)</f>
         <v xml:space="preserve"> </v>
       </c>
     </row>
@@ -1866,17 +1975,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22A42832-12A0-41C9-BED0-20D277223524}">
   <dimension ref="A1:P23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.77734375" customWidth="1"/>
-    <col min="3" max="3" width="24.5546875" customWidth="1"/>
-    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="40.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="24.54296875" customWidth="1"/>
+    <col min="9" max="9" width="14.6328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="40.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
       <c r="F1" t="s">
         <v>0</v>
       </c>
@@ -1911,7 +2020,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>88</v>
       </c>
@@ -1952,10 +2061,17 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>90</v>
       </c>
+      <c r="B3" t="str">
+        <f>_xlfn.XLOOKUP(A3,N2:N10,I2:I10,,1)</f>
+        <v>Angela Martin</v>
+      </c>
+      <c r="C3" t="s">
+        <v>96</v>
+      </c>
       <c r="F3">
         <v>1002</v>
       </c>
@@ -1990,10 +2106,17 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>38</v>
       </c>
+      <c r="B4" t="str">
+        <f>_xlfn.XLOOKUP(A4,N2:N10,I2:I10,,,-1)</f>
+        <v>Michael Scott</v>
+      </c>
+      <c r="C4" t="s">
+        <v>94</v>
+      </c>
       <c r="F4">
         <v>1003</v>
       </c>
@@ -2028,7 +2151,14 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="B5" t="str">
+        <f>_xlfn.XLOOKUP(A4,N2:N10,I2:I10,,,1)</f>
+        <v>Toby Flenderson</v>
+      </c>
+      <c r="C5" t="s">
+        <v>95</v>
+      </c>
       <c r="F5">
         <v>1004</v>
       </c>
@@ -2063,7 +2193,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="F6">
         <v>1005</v>
       </c>
@@ -2098,7 +2228,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="F7">
         <v>1006</v>
       </c>
@@ -2133,7 +2263,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="F8">
         <v>1007</v>
       </c>
@@ -2168,7 +2298,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="F9">
         <v>1008</v>
       </c>
@@ -2203,7 +2333,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="F10">
         <v>1009</v>
       </c>
@@ -2238,15 +2368,15 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="9:9" x14ac:dyDescent="0.35">
       <c r="I22" t="str">
-        <f t="shared" ref="I22:I23" si="0">CONCATENATE(G12," ",H12)</f>
+        <f>CONCATENATE(G12," ",H12)</f>
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="23" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="9:9" x14ac:dyDescent="0.35">
       <c r="I23" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(G13," ",H13)</f>
         <v xml:space="preserve"> </v>
       </c>
     </row>
@@ -2258,12 +2388,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3CCAA7F-6F85-4102-B7D4-D80770622F9F}">
   <dimension ref="A1:S4"/>
-  <sheetFormatPr defaultColWidth="10.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="10.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="7" max="7" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.54296875" customWidth="1"/>
+    <col min="2" max="2" width="15.1796875" customWidth="1"/>
+    <col min="7" max="7" width="12.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B1" t="s">
         <v>73</v>
       </c>
@@ -2304,10 +2436,14 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>70</v>
       </c>
+      <c r="B2">
+        <f>_xlfn.XLOOKUP(I1,H1:S1,H2:S2)</f>
+        <v>310</v>
+      </c>
       <c r="G2" t="s">
         <v>70</v>
       </c>
@@ -2348,10 +2484,14 @@
         <v>288</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>71</v>
       </c>
+      <c r="B3">
+        <f>_xlfn.XLOOKUP(I2,H2:S2,H3:S3)</f>
+        <v>40</v>
+      </c>
       <c r="G3" t="s">
         <v>71</v>
       </c>
@@ -2392,9 +2532,13 @@
         <v>91</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>84</v>
+      </c>
+      <c r="B4">
+        <f t="shared" ref="B4" si="0">_xlfn.XLOOKUP(I3,H3:S3,H4:S4)</f>
+        <v>118</v>
       </c>
       <c r="G4" t="s">
         <v>84</v>
@@ -2443,13 +2587,14 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A2549A4-3A41-4806-B7FD-3B9C6823775F}">
-  <dimension ref="A1:S7"/>
-  <sheetFormatPr defaultColWidth="10.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:S9"/>
+  <sheetFormatPr defaultColWidth="10.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="7" max="7" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.08984375" customWidth="1"/>
+    <col min="7" max="7" width="12.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B1" t="s">
         <v>73</v>
       </c>
@@ -2490,10 +2635,14 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>70</v>
       </c>
+      <c r="B2">
+        <f>_xlfn.XLOOKUP(I1,H1:S1,H2:S2)</f>
+        <v>310</v>
+      </c>
       <c r="G2" t="s">
         <v>70</v>
       </c>
@@ -2534,10 +2683,14 @@
         <v>288</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>71</v>
       </c>
+      <c r="B3">
+        <f>_xlfn.XLOOKUP(I2,H2:S2,H3:S3)</f>
+        <v>40</v>
+      </c>
       <c r="G3" t="s">
         <v>71</v>
       </c>
@@ -2578,10 +2731,14 @@
         <v>91</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>84</v>
       </c>
+      <c r="B4">
+        <f>_xlfn.XLOOKUP(I3,H3:S3,H4:S4)</f>
+        <v>118</v>
+      </c>
       <c r="G4" t="s">
         <v>84</v>
       </c>
@@ -2622,14 +2779,36 @@
         <v>180</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>70</v>
+      </c>
+      <c r="B7">
+        <f>SUM(_xlfn.XLOOKUP(I1,H1:S1,H2:S2):_xlfn.XLOOKUP(J1,H1:S1,H2:S2))</f>
+        <v>460</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8">
+        <f>SUM(_xlfn.XLOOKUP(I2,H2:S2,H3:S3):_xlfn.XLOOKUP(J2,H2:S2,H3:S3))</f>
+        <v>105</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>84</v>
+      </c>
+      <c r="B9">
+        <f>SUM(_xlfn.XLOOKUP(I3,H3:S3,H4:S4):_xlfn.XLOOKUP(J3,H3:S3,H4:S4))</f>
+        <v>263</v>
       </c>
     </row>
   </sheetData>
@@ -2640,12 +2819,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8F9C169-12D8-441E-870D-6C6EF0F6521C}">
   <dimension ref="A1:P10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.44140625" customWidth="1"/>
+    <col min="1" max="1" width="14.453125" customWidth="1"/>
+    <col min="2" max="2" width="28.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
       <c r="E1" t="s">
         <v>0</v>
       </c>
@@ -2664,9 +2844,6 @@
       <c r="J1" t="s">
         <v>4</v>
       </c>
-      <c r="K1" t="s">
-        <v>91</v>
-      </c>
       <c r="L1" t="s">
         <v>5</v>
       </c>
@@ -2683,7 +2860,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>60</v>
       </c>
@@ -2724,10 +2901,14 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>63</v>
       </c>
+      <c r="B3" t="str">
+        <f>VLOOKUP(A3,H2:P10,9,FALSE)</f>
+        <v>Dwight.Schrute@AOL.com</v>
+      </c>
       <c r="E3">
         <v>1002</v>
       </c>
@@ -2762,10 +2943,14 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>66</v>
       </c>
+      <c r="B4" t="str">
+        <f t="shared" ref="B4:B5" si="0">VLOOKUP(A4,H3:P11,8,FALSE)</f>
+        <v>9/11/2013</v>
+      </c>
       <c r="E4">
         <v>1003</v>
       </c>
@@ -2800,10 +2985,14 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>68</v>
       </c>
+      <c r="B5" t="str">
+        <f t="shared" si="0"/>
+        <v>4/22/2015</v>
+      </c>
       <c r="E5">
         <v>1004</v>
       </c>
@@ -2838,7 +3027,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="E6">
         <v>1005</v>
       </c>
@@ -2873,7 +3062,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="E7">
         <v>1006</v>
       </c>
@@ -2908,7 +3097,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="E8">
         <v>1007</v>
       </c>
@@ -2943,7 +3132,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="E9">
         <v>1008</v>
       </c>
@@ -2978,7 +3167,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="E10">
         <v>1009</v>
       </c>

</xml_diff>